<commit_message>
Fixed the Cold Store OSS report notebook
</commit_message>
<xml_diff>
--- a/output/AMIRANTE CCCS - July '26.xlsx
+++ b/output/AMIRANTE CCCS - July '26.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="95">
   <si>
     <t>Date Range:</t>
   </si>
@@ -212,22 +212,19 @@
     <t>location</t>
   </si>
   <si>
-    <t>vessel_client</t>
-  </si>
-  <si>
     <t>date_plugged</t>
   </si>
   <si>
-    <t>time_plugged</t>
-  </si>
-  <si>
     <t>plugged_status</t>
   </si>
   <si>
     <t>date_out</t>
   </si>
   <si>
-    <t>number_of_days_on_plug</t>
+    <t>exit_time</t>
+  </si>
+  <si>
+    <t>days_on_plug</t>
   </si>
   <si>
     <t>set_point</t>
@@ -245,13 +242,34 @@
     <t>storage_price</t>
   </si>
   <si>
+    <t>remarks</t>
+  </si>
+  <si>
+    <t>SUDU6213070</t>
+  </si>
+  <si>
+    <t>Full</t>
+  </si>
+  <si>
+    <t>10:04:00</t>
+  </si>
+  <si>
     <t>SUDU6186817</t>
   </si>
   <si>
-    <t>Full</t>
-  </si>
-  <si>
-    <t>SUDU6213070</t>
+    <t>10:28:00</t>
+  </si>
+  <si>
+    <t>10:25:00</t>
+  </si>
+  <si>
+    <t>14:44:00</t>
+  </si>
+  <si>
+    <t>14:22:00</t>
+  </si>
+  <si>
+    <t>Still On Plug</t>
   </si>
   <si>
     <t>movement_type</t>
@@ -294,17 +312,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00;[Red]-#,##0.00;&quot;-&quot;"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="yyyy-dd-mm"/>
-    <numFmt numFmtId="168" formatCode="#,##0.000;[Red]-#,##0.000"/>
-    <numFmt numFmtId="169" formatCode="#,##0"/>
-    <numFmt numFmtId="170" formatCode="hh:mm:ss;@"/>
-    <numFmt numFmtId="171" formatCode="#,##0;[Red]-#,##0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00;[Red]-#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="169" formatCode="#,##0;[Red]-#,##0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -351,6 +367,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF002060"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF002060"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -379,7 +410,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA9D08E"/>
+        <fgColor rgb="FF006113"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -492,13 +523,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -507,25 +538,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -538,19 +569,19 @@
   <dxfs count="6">
     <dxf/>
     <dxf>
-      <numFmt numFmtId="167" formatCode="yyyy-dd-mm"/>
+      <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="#,##0.000;[Red]-#,##0.000"/>
+      <numFmt numFmtId="165" formatCode="#,##0.00;[Red]-#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="hh:mm:ss;@"/>
+      <numFmt numFmtId="167" formatCode="#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="#,##0"/>
+      <numFmt numFmtId="168" formatCode="yyyy-mm-dd hh:mm"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="171" formatCode="#,##0;[Red]-#,##0"/>
+      <numFmt numFmtId="169" formatCode="#,##0;[Red]-#,##0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -581,10 +612,10 @@
   <tableColumns count="10">
     <tableColumn id="1" name="day_name" dataDxfId="0"/>
     <tableColumn id="2" name="date" dataDxfId="1"/>
-    <tableColumn id="3" name="start_time" dataDxfId="3"/>
+    <tableColumn id="3" name="start_time" dataDxfId="0"/>
     <tableColumn id="4" name="end_time" dataDxfId="0"/>
-    <tableColumn id="5" name="hours" totalsRowFunction="sum" dataDxfId="4"/>
-    <tableColumn id="6" name="overtime_hours" totalsRowFunction="sum" dataDxfId="4"/>
+    <tableColumn id="5" name="hours" totalsRowFunction="sum" dataDxfId="3"/>
+    <tableColumn id="6" name="overtime_hours" totalsRowFunction="sum" dataDxfId="3"/>
     <tableColumn id="7" name="customer" dataDxfId="0"/>
     <tableColumn id="8" name="location" dataDxfId="0"/>
     <tableColumn id="9" name="unit_price" totalsRowFunction="sum" dataDxfId="2"/>
@@ -598,19 +629,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Live_Storage_4" displayName="Live_Storage_4" ref="A1:M9" totalsRowCount="1">
   <autoFilter ref="A1:M8"/>
   <tableColumns count="13">
-    <tableColumn id="1" name="vessel_client" dataDxfId="0"/>
-    <tableColumn id="2" name="date_plugged" dataDxfId="1"/>
-    <tableColumn id="3" name="time_plugged" dataDxfId="3"/>
-    <tableColumn id="4" name="container_number" dataDxfId="0"/>
-    <tableColumn id="5" name="plugged_status" dataDxfId="0"/>
-    <tableColumn id="6" name="date_out" dataDxfId="1"/>
-    <tableColumn id="7" name="number_of_days_on_plug" totalsRowFunction="sum" dataDxfId="5"/>
-    <tableColumn id="8" name="set_point" totalsRowFunction="sum" dataDxfId="5"/>
-    <tableColumn id="9" name="tonnage" totalsRowFunction="sum" dataDxfId="2"/>
-    <tableColumn id="10" name="plugin_price" totalsRowFunction="sum" dataDxfId="2"/>
-    <tableColumn id="11" name="monitoring_price" totalsRowFunction="sum" dataDxfId="2"/>
-    <tableColumn id="12" name="storage_price" totalsRowFunction="sum" dataDxfId="2"/>
-    <tableColumn id="13" name="total_price" totalsRowFunction="sum" dataDxfId="2"/>
+    <tableColumn id="1" name="date_plugged" dataDxfId="4"/>
+    <tableColumn id="2" name="container_number" dataDxfId="0"/>
+    <tableColumn id="3" name="plugged_status" dataDxfId="0"/>
+    <tableColumn id="4" name="date_out" dataDxfId="1"/>
+    <tableColumn id="5" name="exit_time" dataDxfId="0"/>
+    <tableColumn id="6" name="days_on_plug" totalsRowFunction="sum" dataDxfId="5"/>
+    <tableColumn id="7" name="set_point" dataDxfId="0"/>
+    <tableColumn id="8" name="tonnage" totalsRowFunction="sum" dataDxfId="2"/>
+    <tableColumn id="9" name="plugin_price" totalsRowFunction="sum" dataDxfId="2"/>
+    <tableColumn id="10" name="monitoring_price" totalsRowFunction="sum" dataDxfId="2"/>
+    <tableColumn id="11" name="storage_price" totalsRowFunction="sum" dataDxfId="2"/>
+    <tableColumn id="12" name="total_price" totalsRowFunction="sum" dataDxfId="2"/>
+    <tableColumn id="13" name="remarks" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -626,7 +657,7 @@
     <tableColumn id="4" name="movement_type" dataDxfId="0"/>
     <tableColumn id="5" name="destination" dataDxfId="0"/>
     <tableColumn id="6" name="status" dataDxfId="0"/>
-    <tableColumn id="7" name="time_out" dataDxfId="3"/>
+    <tableColumn id="7" name="time_out" dataDxfId="0"/>
     <tableColumn id="8" name="driver" dataDxfId="0"/>
     <tableColumn id="9" name="type" dataDxfId="0"/>
     <tableColumn id="10" name="size" dataDxfId="0"/>
@@ -1063,6 +1094,12 @@
         <v>450</v>
       </c>
     </row>
+    <row r="19" spans="2:7">
+      <c r="D19" s="12"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="13"/>
+    </row>
     <row r="20" spans="2:7">
       <c r="B20" s="11" t="s">
         <v>23</v>
@@ -1119,6 +1156,12 @@
         <v>5</v>
       </c>
     </row>
+    <row r="23" spans="2:7">
+      <c r="D23" s="12"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="13"/>
+    </row>
     <row r="24" spans="2:7">
       <c r="B24" s="11" t="s">
         <v>27</v>
@@ -1137,6 +1180,12 @@
         <v>125</v>
       </c>
     </row>
+    <row r="25" spans="2:7">
+      <c r="D25" s="12"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="13"/>
+    </row>
     <row r="26" spans="2:7">
       <c r="B26" s="11" t="s">
         <v>28</v>
@@ -1154,6 +1203,12 @@
       <c r="G26" s="13">
         <v>150</v>
       </c>
+    </row>
+    <row r="27" spans="2:7">
+      <c r="D27" s="12"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="13"/>
     </row>
     <row r="28" spans="2:7">
       <c r="B28" s="11" t="s">
@@ -1712,18 +1767,19 @@
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
-    <col min="7" max="7" width="24.7109375" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" customWidth="1"/>
-    <col min="11" max="11" width="18.7109375" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" customWidth="1"/>
+    <col min="13" max="13" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1">
@@ -1731,13 +1787,13 @@
         <v>63</v>
       </c>
       <c r="B1" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="D1" s="22" t="s">
         <v>65</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>36</v>
       </c>
       <c r="E1" s="22" t="s">
         <v>66</v>
@@ -1761,321 +1817,303 @@
         <v>72</v>
       </c>
       <c r="L1" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="M1" s="22" t="s">
-        <v>42</v>
-      </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="18">
-        <v>46199</v>
-      </c>
-      <c r="C2" s="23">
-        <v>0.6041666666666666</v>
-      </c>
-      <c r="D2" s="17" t="s">
+      <c r="A2" s="23">
+        <v>46199.44513888889</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>74</v>
       </c>
+      <c r="C2" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="18">
+        <v>46204</v>
+      </c>
       <c r="E2" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="24">
+        <v>1</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="19">
+        <v>0</v>
+      </c>
+      <c r="I2" s="19">
+        <v>0</v>
+      </c>
+      <c r="J2" s="19">
+        <v>30</v>
+      </c>
+      <c r="K2" s="19">
+        <v>70</v>
+      </c>
+      <c r="L2" s="19">
+        <v>100</v>
+      </c>
+      <c r="M2" s="17"/>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="23">
+        <v>46199.60416666666</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F2" s="18">
+      <c r="D3" s="18">
         <v>46204</v>
       </c>
-      <c r="G2" s="24">
+      <c r="E3" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="24">
         <v>1</v>
       </c>
-      <c r="H2" s="24">
-        <v>-25</v>
-      </c>
-      <c r="I2" s="19">
-        <v>28.296</v>
-      </c>
-      <c r="J2" s="19">
-        <v>0</v>
-      </c>
-      <c r="K2" s="19">
+      <c r="G3" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="19">
+        <v>0</v>
+      </c>
+      <c r="I3" s="19">
+        <v>0</v>
+      </c>
+      <c r="J3" s="19">
         <v>30</v>
       </c>
-      <c r="L2" s="19">
+      <c r="K3" s="19">
         <v>70</v>
       </c>
-      <c r="M2" s="19">
+      <c r="L3" s="19">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="18">
-        <v>46199</v>
-      </c>
-      <c r="C3" s="23">
-        <v>0.4451388888888889</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="17" t="s">
+      <c r="M3" s="17"/>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="23">
+        <v>46206.61805555555</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F3" s="18">
-        <v>46204</v>
-      </c>
-      <c r="G3" s="24">
-        <v>1</v>
-      </c>
-      <c r="H3" s="24">
-        <v>-25</v>
-      </c>
-      <c r="I3" s="19">
-        <v>28.476</v>
-      </c>
-      <c r="J3" s="19">
-        <v>0</v>
-      </c>
-      <c r="K3" s="19">
+      <c r="D4" s="18">
+        <v>46211</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" s="24">
+        <v>6</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="19">
+        <v>28.428</v>
+      </c>
+      <c r="I4" s="19">
+        <v>25</v>
+      </c>
+      <c r="J4" s="19">
         <v>30</v>
       </c>
-      <c r="L3" s="19">
-        <v>70</v>
-      </c>
-      <c r="M3" s="19">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="18">
-        <v>46206</v>
-      </c>
-      <c r="C4" s="23">
-        <v>0.6631944444444444</v>
-      </c>
-      <c r="D4" s="17" t="s">
+      <c r="K4" s="19">
+        <v>420</v>
+      </c>
+      <c r="L4" s="19">
+        <v>475</v>
+      </c>
+      <c r="M4" s="17"/>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="23">
+        <v>46206.66319444445</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="C5" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="18">
+      <c r="D5" s="18">
         <v>46211</v>
       </c>
-      <c r="G4" s="24">
+      <c r="E5" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="24">
         <v>6</v>
       </c>
-      <c r="H4" s="24">
-        <v>-25</v>
-      </c>
-      <c r="I4" s="19">
+      <c r="G5" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="19">
         <v>28.977</v>
       </c>
-      <c r="J4" s="19">
+      <c r="I5" s="19">
         <v>25</v>
       </c>
-      <c r="K4" s="19">
+      <c r="J5" s="19">
         <v>30</v>
       </c>
-      <c r="L4" s="19">
+      <c r="K5" s="19">
         <v>420</v>
       </c>
-      <c r="M4" s="19">
+      <c r="L5" s="19">
         <v>475</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="18">
-        <v>46206</v>
-      </c>
-      <c r="C5" s="23">
-        <v>0.7097222222222223</v>
-      </c>
-      <c r="D5" s="17" t="s">
+      <c r="M5" s="17"/>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="23">
+        <v>46206.70972222222</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="C6" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F5" s="18">
+      <c r="D6" s="18">
         <v>46211</v>
       </c>
-      <c r="G5" s="24">
+      <c r="E6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="24">
         <v>6</v>
       </c>
-      <c r="H5" s="24">
-        <v>-25</v>
-      </c>
-      <c r="I5" s="19">
+      <c r="G6" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="19">
         <v>28.461</v>
       </c>
-      <c r="J5" s="19">
+      <c r="I6" s="19">
         <v>25</v>
       </c>
-      <c r="K5" s="19">
+      <c r="J6" s="19">
         <v>30</v>
       </c>
-      <c r="L5" s="19">
+      <c r="K6" s="19">
         <v>420</v>
       </c>
-      <c r="M5" s="19">
+      <c r="L6" s="19">
         <v>475</v>
       </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="18">
-        <v>46206</v>
-      </c>
-      <c r="C6" s="23">
-        <v>0.6180555555555556</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="17" t="s">
+      <c r="M6" s="17"/>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="23">
+        <v>46210.6125</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F6" s="18">
-        <v>46211</v>
-      </c>
-      <c r="G6" s="24">
-        <v>6</v>
-      </c>
-      <c r="H6" s="24">
-        <v>-25</v>
-      </c>
-      <c r="I6" s="19">
-        <v>28.428</v>
-      </c>
-      <c r="J6" s="19">
+      <c r="D7" s="18"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="24">
         <v>25</v>
       </c>
-      <c r="K6" s="19">
-        <v>30</v>
-      </c>
-      <c r="L6" s="19">
-        <v>420</v>
-      </c>
-      <c r="M6" s="19">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="18">
-        <v>46210</v>
-      </c>
-      <c r="C7" s="23">
-        <v>0.6145833333333334</v>
-      </c>
-      <c r="D7" s="17" t="s">
+      <c r="G7" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="19">
+        <v>28.567</v>
+      </c>
+      <c r="I7" s="19">
+        <v>25</v>
+      </c>
+      <c r="J7" s="19">
+        <v>0</v>
+      </c>
+      <c r="K7" s="19">
+        <v>1750</v>
+      </c>
+      <c r="L7" s="19">
+        <v>1775</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="23">
+        <v>46210.61458333334</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="C8" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="24">
+      <c r="D8" s="18"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="24">
         <v>25</v>
       </c>
-      <c r="H7" s="24">
-        <v>-25</v>
-      </c>
-      <c r="I7" s="19">
+      <c r="G8" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="19">
         <v>28.278</v>
       </c>
-      <c r="J7" s="19">
+      <c r="I8" s="19">
         <v>25</v>
       </c>
-      <c r="K7" s="19">
-        <v>0</v>
-      </c>
-      <c r="L7" s="19">
+      <c r="J8" s="19">
+        <v>0</v>
+      </c>
+      <c r="K8" s="19">
         <v>1750</v>
       </c>
-      <c r="M7" s="19">
+      <c r="L8" s="19">
         <v>1775</v>
       </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="18">
-        <v>46210</v>
-      </c>
-      <c r="C8" s="23">
-        <v>0.6125</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="24">
-        <v>25</v>
-      </c>
-      <c r="H8" s="24">
-        <v>-25</v>
-      </c>
-      <c r="I8" s="19">
-        <v>28.567</v>
-      </c>
-      <c r="J8" s="19">
-        <v>25</v>
-      </c>
-      <c r="K8" s="19">
-        <v>0</v>
-      </c>
-      <c r="L8" s="19">
-        <v>1750</v>
-      </c>
-      <c r="M8" s="19">
-        <v>1775</v>
+      <c r="M8" s="17" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="G9" s="24">
-        <f>SUBTOTAL(109,[number_of_days_on_plug])</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="24">
-        <f>SUBTOTAL(109,[set_point])</f>
+      <c r="F9" s="24">
+        <f>SUBTOTAL(109,[days_on_plug])</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="19">
+        <f>SUBTOTAL(109,[tonnage])</f>
         <v>0</v>
       </c>
       <c r="I9" s="19">
-        <f>SUBTOTAL(109,[tonnage])</f>
+        <f>SUBTOTAL(109,[plugin_price])</f>
         <v>0</v>
       </c>
       <c r="J9" s="19">
-        <f>SUBTOTAL(109,[plugin_price])</f>
+        <f>SUBTOTAL(109,[monitoring_price])</f>
         <v>0</v>
       </c>
       <c r="K9" s="19">
-        <f>SUBTOTAL(109,[monitoring_price])</f>
+        <f>SUBTOTAL(109,[storage_price])</f>
         <v>0</v>
       </c>
       <c r="L9" s="19">
-        <f>SUBTOTAL(109,[storage_price])</f>
-        <v>0</v>
-      </c>
-      <c r="M9" s="19">
         <f>SUBTOTAL(109,[total_price])</f>
         <v>0</v>
       </c>
@@ -2126,31 +2164,31 @@
         <v>35</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G1" s="25" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H1" s="25" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="J1" s="25" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="K1" s="25" t="s">
         <v>37</v>
       </c>
       <c r="L1" s="25" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2158,28 +2196,28 @@
         <v>52</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="C2" s="18">
-        <v>46211</v>
+        <v>46204</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="G2" s="23">
-        <v>0.4340277777777778</v>
+      <c r="G2" s="17" t="s">
+        <v>76</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="J2" s="17" t="s">
         <v>21</v>
@@ -2196,28 +2234,28 @@
         <v>52</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3" s="18">
         <v>46204</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="G3" s="23">
-        <v>0.4194444444444445</v>
+      <c r="G3" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="J3" s="17" t="s">
         <v>21</v>
@@ -2234,28 +2272,28 @@
         <v>52</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="C4" s="18">
-        <v>46204</v>
+        <v>46211</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="G4" s="23">
-        <v>0.4361111111111111</v>
+      <c r="G4" s="17" t="s">
+        <v>81</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>21</v>
@@ -2272,28 +2310,28 @@
         <v>52</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C5" s="18">
         <v>46211</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="23">
-        <v>0.5986111111111111</v>
+      <c r="G5" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I5" s="17" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="J5" s="17" t="s">
         <v>21</v>
@@ -2310,28 +2348,28 @@
         <v>52</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C6" s="18">
         <v>46211</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="G6" s="23">
-        <v>0.6138888888888889</v>
+      <c r="G6" s="17" t="s">
+        <v>79</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="J6" s="17" t="s">
         <v>21</v>

</xml_diff>